<commit_message>
tesztelés, dokumentálás, kód rendezés
-dokumentáció írás
-output generálás
-hónapok data_table-be helyezése
-kötvény és babakötvény feltételes plot-ra helyezése
</commit_message>
<xml_diff>
--- a/python/penzugy_vizualizator/konyveles.xlsx
+++ b/python/penzugy_vizualizator/konyveles.xlsx
@@ -1,20 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="20417"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="H:\IT\Github Projects\python\penzugy_vizualizator\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\koppany.balazs.endre\Documents\GitHub\github_projects\Github Projects\python\penzugy_vizualizator\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF524E05-7E86-4D7D-AA07-DB87E392CA14}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="20400" windowHeight="7620" tabRatio="500"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="20400" windowHeight="7620" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="2026" sheetId="4" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913" iterateDelta="1E-4"/>
+  <calcPr calcId="191029" iterateDelta="1E-4"/>
   <extLst>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
       <loext:extCalcPr stringRefSyntax="ExcelA1"/>
@@ -203,7 +204,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="#,##0&quot; Ft&quot;"/>
   </numFmts>
@@ -697,16 +698,16 @@
     <xf numFmtId="164" fontId="0" fillId="10" borderId="8" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -973,7 +974,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:FN17"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1096,18 +1097,18 @@
       <c r="D1" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="E1" s="59" t="s">
+      <c r="E1" s="56" t="s">
         <v>11</v>
       </c>
-      <c r="F1" s="59"/>
-      <c r="G1" s="59"/>
-      <c r="H1" s="59"/>
-      <c r="I1" s="59"/>
-      <c r="J1" s="59"/>
-      <c r="K1" s="59"/>
-      <c r="L1" s="59"/>
-      <c r="M1" s="59"/>
-      <c r="N1" s="59"/>
+      <c r="F1" s="56"/>
+      <c r="G1" s="56"/>
+      <c r="H1" s="56"/>
+      <c r="I1" s="56"/>
+      <c r="J1" s="56"/>
+      <c r="K1" s="56"/>
+      <c r="L1" s="56"/>
+      <c r="M1" s="56"/>
+      <c r="N1" s="56"/>
       <c r="O1" s="3" t="s">
         <v>23</v>
       </c>
@@ -1117,18 +1118,18 @@
       <c r="R1" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="S1" s="59" t="s">
+      <c r="S1" s="56" t="s">
         <v>12</v>
       </c>
-      <c r="T1" s="59"/>
-      <c r="U1" s="59"/>
-      <c r="V1" s="59"/>
-      <c r="W1" s="59"/>
-      <c r="X1" s="59"/>
-      <c r="Y1" s="59"/>
-      <c r="Z1" s="59"/>
-      <c r="AA1" s="59"/>
-      <c r="AB1" s="59"/>
+      <c r="T1" s="56"/>
+      <c r="U1" s="56"/>
+      <c r="V1" s="56"/>
+      <c r="W1" s="56"/>
+      <c r="X1" s="56"/>
+      <c r="Y1" s="56"/>
+      <c r="Z1" s="56"/>
+      <c r="AA1" s="56"/>
+      <c r="AB1" s="56"/>
       <c r="AC1" s="3" t="s">
         <v>23</v>
       </c>
@@ -1138,18 +1139,18 @@
       <c r="AF1" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="AG1" s="59" t="s">
+      <c r="AG1" s="56" t="s">
         <v>13</v>
       </c>
-      <c r="AH1" s="59"/>
-      <c r="AI1" s="59"/>
-      <c r="AJ1" s="59"/>
-      <c r="AK1" s="59"/>
-      <c r="AL1" s="59"/>
-      <c r="AM1" s="59"/>
-      <c r="AN1" s="59"/>
-      <c r="AO1" s="59"/>
-      <c r="AP1" s="59"/>
+      <c r="AH1" s="56"/>
+      <c r="AI1" s="56"/>
+      <c r="AJ1" s="56"/>
+      <c r="AK1" s="56"/>
+      <c r="AL1" s="56"/>
+      <c r="AM1" s="56"/>
+      <c r="AN1" s="56"/>
+      <c r="AO1" s="56"/>
+      <c r="AP1" s="56"/>
       <c r="AQ1" s="3" t="s">
         <v>23</v>
       </c>
@@ -1159,18 +1160,18 @@
       <c r="AT1" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="AU1" s="59" t="s">
+      <c r="AU1" s="56" t="s">
         <v>2</v>
       </c>
-      <c r="AV1" s="59"/>
-      <c r="AW1" s="59"/>
-      <c r="AX1" s="59"/>
-      <c r="AY1" s="59"/>
-      <c r="AZ1" s="59"/>
-      <c r="BA1" s="59"/>
-      <c r="BB1" s="59"/>
-      <c r="BC1" s="59"/>
-      <c r="BD1" s="59"/>
+      <c r="AV1" s="56"/>
+      <c r="AW1" s="56"/>
+      <c r="AX1" s="56"/>
+      <c r="AY1" s="56"/>
+      <c r="AZ1" s="56"/>
+      <c r="BA1" s="56"/>
+      <c r="BB1" s="56"/>
+      <c r="BC1" s="56"/>
+      <c r="BD1" s="56"/>
       <c r="BE1" s="3" t="s">
         <v>23</v>
       </c>
@@ -1180,18 +1181,18 @@
       <c r="BH1" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="BI1" s="59" t="s">
+      <c r="BI1" s="56" t="s">
         <v>3</v>
       </c>
-      <c r="BJ1" s="59"/>
-      <c r="BK1" s="59"/>
-      <c r="BL1" s="59"/>
-      <c r="BM1" s="59"/>
-      <c r="BN1" s="59"/>
-      <c r="BO1" s="59"/>
-      <c r="BP1" s="59"/>
-      <c r="BQ1" s="59"/>
-      <c r="BR1" s="59"/>
+      <c r="BJ1" s="56"/>
+      <c r="BK1" s="56"/>
+      <c r="BL1" s="56"/>
+      <c r="BM1" s="56"/>
+      <c r="BN1" s="56"/>
+      <c r="BO1" s="56"/>
+      <c r="BP1" s="56"/>
+      <c r="BQ1" s="56"/>
+      <c r="BR1" s="56"/>
       <c r="BS1" s="3" t="s">
         <v>23</v>
       </c>
@@ -1201,18 +1202,18 @@
       <c r="BV1" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="BW1" s="59" t="s">
+      <c r="BW1" s="56" t="s">
         <v>4</v>
       </c>
-      <c r="BX1" s="59"/>
-      <c r="BY1" s="59"/>
-      <c r="BZ1" s="59"/>
-      <c r="CA1" s="59"/>
-      <c r="CB1" s="59"/>
-      <c r="CC1" s="59"/>
-      <c r="CD1" s="59"/>
-      <c r="CE1" s="59"/>
-      <c r="CF1" s="59"/>
+      <c r="BX1" s="56"/>
+      <c r="BY1" s="56"/>
+      <c r="BZ1" s="56"/>
+      <c r="CA1" s="56"/>
+      <c r="CB1" s="56"/>
+      <c r="CC1" s="56"/>
+      <c r="CD1" s="56"/>
+      <c r="CE1" s="56"/>
+      <c r="CF1" s="56"/>
       <c r="CG1" s="3" t="s">
         <v>23</v>
       </c>
@@ -1222,18 +1223,18 @@
       <c r="CJ1" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="CK1" s="59" t="s">
+      <c r="CK1" s="56" t="s">
         <v>5</v>
       </c>
-      <c r="CL1" s="59"/>
-      <c r="CM1" s="59"/>
-      <c r="CN1" s="59"/>
-      <c r="CO1" s="59"/>
-      <c r="CP1" s="59"/>
-      <c r="CQ1" s="59"/>
-      <c r="CR1" s="59"/>
-      <c r="CS1" s="59"/>
-      <c r="CT1" s="59"/>
+      <c r="CL1" s="56"/>
+      <c r="CM1" s="56"/>
+      <c r="CN1" s="56"/>
+      <c r="CO1" s="56"/>
+      <c r="CP1" s="56"/>
+      <c r="CQ1" s="56"/>
+      <c r="CR1" s="56"/>
+      <c r="CS1" s="56"/>
+      <c r="CT1" s="56"/>
       <c r="CU1" s="3" t="s">
         <v>23</v>
       </c>
@@ -1243,18 +1244,18 @@
       <c r="CX1" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="CY1" s="59" t="s">
+      <c r="CY1" s="56" t="s">
         <v>6</v>
       </c>
-      <c r="CZ1" s="59"/>
-      <c r="DA1" s="59"/>
-      <c r="DB1" s="59"/>
-      <c r="DC1" s="59"/>
-      <c r="DD1" s="59"/>
-      <c r="DE1" s="59"/>
-      <c r="DF1" s="59"/>
-      <c r="DG1" s="59"/>
-      <c r="DH1" s="59"/>
+      <c r="CZ1" s="56"/>
+      <c r="DA1" s="56"/>
+      <c r="DB1" s="56"/>
+      <c r="DC1" s="56"/>
+      <c r="DD1" s="56"/>
+      <c r="DE1" s="56"/>
+      <c r="DF1" s="56"/>
+      <c r="DG1" s="56"/>
+      <c r="DH1" s="56"/>
       <c r="DI1" s="3" t="s">
         <v>23</v>
       </c>
@@ -1264,18 +1265,18 @@
       <c r="DL1" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="DM1" s="59" t="s">
+      <c r="DM1" s="56" t="s">
         <v>7</v>
       </c>
-      <c r="DN1" s="59"/>
-      <c r="DO1" s="59"/>
-      <c r="DP1" s="59"/>
-      <c r="DQ1" s="59"/>
-      <c r="DR1" s="59"/>
-      <c r="DS1" s="59"/>
-      <c r="DT1" s="59"/>
-      <c r="DU1" s="59"/>
-      <c r="DV1" s="59"/>
+      <c r="DN1" s="56"/>
+      <c r="DO1" s="56"/>
+      <c r="DP1" s="56"/>
+      <c r="DQ1" s="56"/>
+      <c r="DR1" s="56"/>
+      <c r="DS1" s="56"/>
+      <c r="DT1" s="56"/>
+      <c r="DU1" s="56"/>
+      <c r="DV1" s="56"/>
       <c r="DW1" s="3" t="s">
         <v>23</v>
       </c>
@@ -1285,18 +1286,18 @@
       <c r="DZ1" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="EA1" s="59" t="s">
+      <c r="EA1" s="56" t="s">
         <v>8</v>
       </c>
-      <c r="EB1" s="59"/>
-      <c r="EC1" s="59"/>
-      <c r="ED1" s="59"/>
-      <c r="EE1" s="59"/>
-      <c r="EF1" s="59"/>
-      <c r="EG1" s="59"/>
-      <c r="EH1" s="59"/>
-      <c r="EI1" s="59"/>
-      <c r="EJ1" s="59"/>
+      <c r="EB1" s="56"/>
+      <c r="EC1" s="56"/>
+      <c r="ED1" s="56"/>
+      <c r="EE1" s="56"/>
+      <c r="EF1" s="56"/>
+      <c r="EG1" s="56"/>
+      <c r="EH1" s="56"/>
+      <c r="EI1" s="56"/>
+      <c r="EJ1" s="56"/>
       <c r="EK1" s="3" t="s">
         <v>23</v>
       </c>
@@ -1306,18 +1307,18 @@
       <c r="EN1" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="EO1" s="59" t="s">
+      <c r="EO1" s="56" t="s">
         <v>9</v>
       </c>
-      <c r="EP1" s="59"/>
-      <c r="EQ1" s="59"/>
-      <c r="ER1" s="59"/>
-      <c r="ES1" s="59"/>
-      <c r="ET1" s="59"/>
-      <c r="EU1" s="59"/>
-      <c r="EV1" s="59"/>
-      <c r="EW1" s="59"/>
-      <c r="EX1" s="59"/>
+      <c r="EP1" s="56"/>
+      <c r="EQ1" s="56"/>
+      <c r="ER1" s="56"/>
+      <c r="ES1" s="56"/>
+      <c r="ET1" s="56"/>
+      <c r="EU1" s="56"/>
+      <c r="EV1" s="56"/>
+      <c r="EW1" s="56"/>
+      <c r="EX1" s="56"/>
       <c r="EY1" s="3" t="s">
         <v>23</v>
       </c>
@@ -1327,18 +1328,18 @@
       <c r="FB1" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="FC1" s="59" t="s">
+      <c r="FC1" s="56" t="s">
         <v>10</v>
       </c>
-      <c r="FD1" s="59"/>
-      <c r="FE1" s="59"/>
-      <c r="FF1" s="59"/>
-      <c r="FG1" s="59"/>
-      <c r="FH1" s="59"/>
-      <c r="FI1" s="59"/>
-      <c r="FJ1" s="59"/>
-      <c r="FK1" s="59"/>
-      <c r="FL1" s="59"/>
+      <c r="FD1" s="56"/>
+      <c r="FE1" s="56"/>
+      <c r="FF1" s="56"/>
+      <c r="FG1" s="56"/>
+      <c r="FH1" s="56"/>
+      <c r="FI1" s="56"/>
+      <c r="FJ1" s="56"/>
+      <c r="FK1" s="56"/>
+      <c r="FL1" s="56"/>
       <c r="FM1" s="3" t="s">
         <v>23</v>
       </c>
@@ -1355,22 +1356,22 @@
       <c r="D2" s="8">
         <v>2061000</v>
       </c>
-      <c r="E2" s="58" t="s">
+      <c r="E2" s="57" t="s">
         <v>18</v>
       </c>
-      <c r="F2" s="58"/>
-      <c r="G2" s="56" t="s">
+      <c r="F2" s="57"/>
+      <c r="G2" s="58" t="s">
         <v>14</v>
       </c>
-      <c r="H2" s="56"/>
-      <c r="I2" s="56"/>
-      <c r="J2" s="56"/>
-      <c r="K2" s="57" t="s">
+      <c r="H2" s="58"/>
+      <c r="I2" s="58"/>
+      <c r="J2" s="58"/>
+      <c r="K2" s="59" t="s">
         <v>15</v>
       </c>
-      <c r="L2" s="57"/>
-      <c r="M2" s="57"/>
-      <c r="N2" s="57"/>
+      <c r="L2" s="59"/>
+      <c r="M2" s="59"/>
+      <c r="N2" s="59"/>
       <c r="O2" s="9">
         <f>45000+G17-I17</f>
         <v>40010</v>
@@ -1382,22 +1383,22 @@
         <f>O6</f>
         <v>2111900</v>
       </c>
-      <c r="S2" s="58" t="s">
+      <c r="S2" s="57" t="s">
         <v>18</v>
       </c>
-      <c r="T2" s="58"/>
-      <c r="U2" s="56" t="s">
+      <c r="T2" s="57"/>
+      <c r="U2" s="58" t="s">
         <v>14</v>
       </c>
-      <c r="V2" s="56"/>
-      <c r="W2" s="56"/>
-      <c r="X2" s="56"/>
-      <c r="Y2" s="57" t="s">
+      <c r="V2" s="58"/>
+      <c r="W2" s="58"/>
+      <c r="X2" s="58"/>
+      <c r="Y2" s="59" t="s">
         <v>15</v>
       </c>
-      <c r="Z2" s="57"/>
-      <c r="AA2" s="57"/>
-      <c r="AB2" s="57"/>
+      <c r="Z2" s="59"/>
+      <c r="AA2" s="59"/>
+      <c r="AB2" s="59"/>
       <c r="AC2" s="9">
         <f>O2+U17-W17</f>
         <v>36920</v>
@@ -1409,22 +1410,22 @@
         <f>AC6</f>
         <v>2162210</v>
       </c>
-      <c r="AG2" s="58" t="s">
+      <c r="AG2" s="57" t="s">
         <v>18</v>
       </c>
-      <c r="AH2" s="58"/>
-      <c r="AI2" s="56" t="s">
+      <c r="AH2" s="57"/>
+      <c r="AI2" s="58" t="s">
         <v>14</v>
       </c>
-      <c r="AJ2" s="56"/>
-      <c r="AK2" s="56"/>
-      <c r="AL2" s="56"/>
-      <c r="AM2" s="57" t="s">
+      <c r="AJ2" s="58"/>
+      <c r="AK2" s="58"/>
+      <c r="AL2" s="58"/>
+      <c r="AM2" s="59" t="s">
         <v>15</v>
       </c>
-      <c r="AN2" s="57"/>
-      <c r="AO2" s="57"/>
-      <c r="AP2" s="57"/>
+      <c r="AN2" s="59"/>
+      <c r="AO2" s="59"/>
+      <c r="AP2" s="59"/>
       <c r="AQ2" s="9">
         <f>AC2+AI17-AK17</f>
         <v>38030</v>
@@ -1436,22 +1437,22 @@
         <f>AQ6</f>
         <v>2215620</v>
       </c>
-      <c r="AU2" s="58" t="s">
+      <c r="AU2" s="57" t="s">
         <v>18</v>
       </c>
-      <c r="AV2" s="58"/>
-      <c r="AW2" s="56" t="s">
+      <c r="AV2" s="57"/>
+      <c r="AW2" s="58" t="s">
         <v>14</v>
       </c>
-      <c r="AX2" s="56"/>
-      <c r="AY2" s="56"/>
-      <c r="AZ2" s="56"/>
-      <c r="BA2" s="57" t="s">
+      <c r="AX2" s="58"/>
+      <c r="AY2" s="58"/>
+      <c r="AZ2" s="58"/>
+      <c r="BA2" s="59" t="s">
         <v>15</v>
       </c>
-      <c r="BB2" s="57"/>
-      <c r="BC2" s="57"/>
-      <c r="BD2" s="57"/>
+      <c r="BB2" s="59"/>
+      <c r="BC2" s="59"/>
+      <c r="BD2" s="59"/>
       <c r="BE2" s="9">
         <f>AQ2+AW17-AY17</f>
         <v>34940</v>
@@ -1463,22 +1464,22 @@
         <f>BE6</f>
         <v>2261630</v>
       </c>
-      <c r="BI2" s="58" t="s">
+      <c r="BI2" s="57" t="s">
         <v>18</v>
       </c>
-      <c r="BJ2" s="58"/>
-      <c r="BK2" s="56" t="s">
+      <c r="BJ2" s="57"/>
+      <c r="BK2" s="58" t="s">
         <v>14</v>
       </c>
-      <c r="BL2" s="56"/>
-      <c r="BM2" s="56"/>
-      <c r="BN2" s="56"/>
-      <c r="BO2" s="57" t="s">
+      <c r="BL2" s="58"/>
+      <c r="BM2" s="58"/>
+      <c r="BN2" s="58"/>
+      <c r="BO2" s="59" t="s">
         <v>15</v>
       </c>
-      <c r="BP2" s="57"/>
-      <c r="BQ2" s="57"/>
-      <c r="BR2" s="57"/>
+      <c r="BP2" s="59"/>
+      <c r="BQ2" s="59"/>
+      <c r="BR2" s="59"/>
       <c r="BS2" s="9">
         <f>BE2+BK17-BM17</f>
         <v>51950</v>
@@ -1490,22 +1491,22 @@
         <f>BS6</f>
         <v>2318540</v>
       </c>
-      <c r="BW2" s="58" t="s">
+      <c r="BW2" s="57" t="s">
         <v>18</v>
       </c>
-      <c r="BX2" s="58"/>
-      <c r="BY2" s="56" t="s">
+      <c r="BX2" s="57"/>
+      <c r="BY2" s="58" t="s">
         <v>14</v>
       </c>
-      <c r="BZ2" s="56"/>
-      <c r="CA2" s="56"/>
-      <c r="CB2" s="56"/>
-      <c r="CC2" s="57" t="s">
+      <c r="BZ2" s="58"/>
+      <c r="CA2" s="58"/>
+      <c r="CB2" s="58"/>
+      <c r="CC2" s="59" t="s">
         <v>15</v>
       </c>
-      <c r="CD2" s="57"/>
-      <c r="CE2" s="57"/>
-      <c r="CF2" s="57"/>
+      <c r="CD2" s="59"/>
+      <c r="CE2" s="59"/>
+      <c r="CF2" s="59"/>
       <c r="CG2" s="9">
         <f>BS2+BY17-CA17</f>
         <v>48460</v>
@@ -1517,22 +1518,22 @@
         <f>CG6</f>
         <v>2483750</v>
       </c>
-      <c r="CK2" s="58" t="s">
+      <c r="CK2" s="57" t="s">
         <v>18</v>
       </c>
-      <c r="CL2" s="58"/>
-      <c r="CM2" s="56" t="s">
+      <c r="CL2" s="57"/>
+      <c r="CM2" s="58" t="s">
         <v>14</v>
       </c>
-      <c r="CN2" s="56"/>
-      <c r="CO2" s="56"/>
-      <c r="CP2" s="56"/>
-      <c r="CQ2" s="57" t="s">
+      <c r="CN2" s="58"/>
+      <c r="CO2" s="58"/>
+      <c r="CP2" s="58"/>
+      <c r="CQ2" s="59" t="s">
         <v>15</v>
       </c>
-      <c r="CR2" s="57"/>
-      <c r="CS2" s="57"/>
-      <c r="CT2" s="57"/>
+      <c r="CR2" s="59"/>
+      <c r="CS2" s="59"/>
+      <c r="CT2" s="59"/>
       <c r="CU2" s="9">
         <f>CG2+CM17-CO17</f>
         <v>46660</v>
@@ -1544,22 +1545,22 @@
         <f>CU6</f>
         <v>2464550</v>
       </c>
-      <c r="CY2" s="58" t="s">
+      <c r="CY2" s="57" t="s">
         <v>18</v>
       </c>
-      <c r="CZ2" s="58"/>
-      <c r="DA2" s="56" t="s">
+      <c r="CZ2" s="57"/>
+      <c r="DA2" s="58" t="s">
         <v>14</v>
       </c>
-      <c r="DB2" s="56"/>
-      <c r="DC2" s="56"/>
-      <c r="DD2" s="56"/>
-      <c r="DE2" s="57" t="s">
+      <c r="DB2" s="58"/>
+      <c r="DC2" s="58"/>
+      <c r="DD2" s="58"/>
+      <c r="DE2" s="59" t="s">
         <v>15</v>
       </c>
-      <c r="DF2" s="57"/>
-      <c r="DG2" s="57"/>
-      <c r="DH2" s="57"/>
+      <c r="DF2" s="59"/>
+      <c r="DG2" s="59"/>
+      <c r="DH2" s="59"/>
       <c r="DI2" s="9">
         <f>CU2+DA17-DC17</f>
         <v>44860</v>
@@ -1571,22 +1572,22 @@
         <f>DI6</f>
         <v>2341750</v>
       </c>
-      <c r="DM2" s="58" t="s">
+      <c r="DM2" s="57" t="s">
         <v>18</v>
       </c>
-      <c r="DN2" s="58"/>
-      <c r="DO2" s="56" t="s">
+      <c r="DN2" s="57"/>
+      <c r="DO2" s="58" t="s">
         <v>14</v>
       </c>
-      <c r="DP2" s="56"/>
-      <c r="DQ2" s="56"/>
-      <c r="DR2" s="56"/>
-      <c r="DS2" s="57" t="s">
+      <c r="DP2" s="58"/>
+      <c r="DQ2" s="58"/>
+      <c r="DR2" s="58"/>
+      <c r="DS2" s="59" t="s">
         <v>15</v>
       </c>
-      <c r="DT2" s="57"/>
-      <c r="DU2" s="57"/>
-      <c r="DV2" s="57"/>
+      <c r="DT2" s="59"/>
+      <c r="DU2" s="59"/>
+      <c r="DV2" s="59"/>
       <c r="DW2" s="9">
         <f>DI2+DO17-DQ17</f>
         <v>26870</v>
@@ -1598,22 +1599,22 @@
         <f>DW6</f>
         <v>2358860</v>
       </c>
-      <c r="EA2" s="58" t="s">
+      <c r="EA2" s="57" t="s">
         <v>18</v>
       </c>
-      <c r="EB2" s="58"/>
-      <c r="EC2" s="56" t="s">
+      <c r="EB2" s="57"/>
+      <c r="EC2" s="58" t="s">
         <v>14</v>
       </c>
-      <c r="ED2" s="56"/>
-      <c r="EE2" s="56"/>
-      <c r="EF2" s="56"/>
-      <c r="EG2" s="57" t="s">
+      <c r="ED2" s="58"/>
+      <c r="EE2" s="58"/>
+      <c r="EF2" s="58"/>
+      <c r="EG2" s="59" t="s">
         <v>15</v>
       </c>
-      <c r="EH2" s="57"/>
-      <c r="EI2" s="57"/>
-      <c r="EJ2" s="57"/>
+      <c r="EH2" s="59"/>
+      <c r="EI2" s="59"/>
+      <c r="EJ2" s="59"/>
       <c r="EK2" s="9">
         <f>DW2+EC17-EE17</f>
         <v>24180</v>
@@ -1623,24 +1624,24 @@
       </c>
       <c r="EN2" s="8">
         <f>EK6</f>
-        <v>2283470</v>
-      </c>
-      <c r="EO2" s="58" t="s">
+        <v>2413470</v>
+      </c>
+      <c r="EO2" s="57" t="s">
         <v>18</v>
       </c>
-      <c r="EP2" s="58"/>
-      <c r="EQ2" s="56" t="s">
+      <c r="EP2" s="57"/>
+      <c r="EQ2" s="58" t="s">
         <v>14</v>
       </c>
-      <c r="ER2" s="56"/>
-      <c r="ES2" s="56"/>
-      <c r="ET2" s="56"/>
-      <c r="EU2" s="57" t="s">
+      <c r="ER2" s="58"/>
+      <c r="ES2" s="58"/>
+      <c r="ET2" s="58"/>
+      <c r="EU2" s="59" t="s">
         <v>15</v>
       </c>
-      <c r="EV2" s="57"/>
-      <c r="EW2" s="57"/>
-      <c r="EX2" s="57"/>
+      <c r="EV2" s="59"/>
+      <c r="EW2" s="59"/>
+      <c r="EX2" s="59"/>
       <c r="EY2" s="9">
         <f>EK2+EQ17-ES17</f>
         <v>20890</v>
@@ -1650,24 +1651,24 @@
       </c>
       <c r="FB2" s="8">
         <f>EY6</f>
-        <v>2338980</v>
-      </c>
-      <c r="FC2" s="58" t="s">
+        <v>2468980</v>
+      </c>
+      <c r="FC2" s="57" t="s">
         <v>18</v>
       </c>
-      <c r="FD2" s="58"/>
-      <c r="FE2" s="56" t="s">
+      <c r="FD2" s="57"/>
+      <c r="FE2" s="58" t="s">
         <v>14</v>
       </c>
-      <c r="FF2" s="56"/>
-      <c r="FG2" s="56"/>
-      <c r="FH2" s="56"/>
-      <c r="FI2" s="57" t="s">
+      <c r="FF2" s="58"/>
+      <c r="FG2" s="58"/>
+      <c r="FH2" s="58"/>
+      <c r="FI2" s="59" t="s">
         <v>15</v>
       </c>
-      <c r="FJ2" s="57"/>
-      <c r="FK2" s="57"/>
-      <c r="FL2" s="57"/>
+      <c r="FJ2" s="59"/>
+      <c r="FK2" s="59"/>
+      <c r="FL2" s="59"/>
       <c r="FM2" s="9">
         <f>EY2+FE17-FG17</f>
         <v>27000</v>
@@ -2842,8 +2843,8 @@
         <v>36</v>
       </c>
       <c r="EK5" s="18">
-        <f>DW5</f>
-        <v>2120000</v>
+        <f>DW5+130000</f>
+        <v>2250000</v>
       </c>
       <c r="EL5" s="19" t="s">
         <v>37</v>
@@ -2873,7 +2874,7 @@
       </c>
       <c r="EY5" s="18">
         <f>EK5+45000</f>
-        <v>2165000</v>
+        <v>2295000</v>
       </c>
       <c r="EZ5" s="19" t="s">
         <v>37</v>
@@ -2907,7 +2908,7 @@
       </c>
       <c r="FM5" s="18">
         <f>EY5</f>
-        <v>2165000</v>
+        <v>2295000</v>
       </c>
       <c r="FN5" s="19" t="s">
         <v>37</v>
@@ -3129,7 +3130,7 @@
       </c>
       <c r="EK6" s="18">
         <f>SUM(EK2:EK5)</f>
-        <v>2283470</v>
+        <v>2413470</v>
       </c>
       <c r="EL6" s="19" t="s">
         <v>17</v>
@@ -3151,7 +3152,7 @@
       </c>
       <c r="EY6" s="18">
         <f>SUM(EY2:EY5)</f>
-        <v>2338980</v>
+        <v>2468980</v>
       </c>
       <c r="EZ6" s="19" t="s">
         <v>17</v>
@@ -3177,7 +3178,7 @@
       </c>
       <c r="FM6" s="18">
         <f>SUM(FM2:FM5)</f>
-        <v>2374290</v>
+        <v>2504290</v>
       </c>
       <c r="FN6" s="19" t="s">
         <v>17</v>
@@ -3593,7 +3594,7 @@
       <c r="EJ8" s="3"/>
       <c r="EK8" s="39">
         <f>EK6-DZ2</f>
-        <v>-75390</v>
+        <v>54610</v>
       </c>
       <c r="EL8" s="38" t="s">
         <v>46</v>
@@ -5396,16 +5397,28 @@
     </row>
   </sheetData>
   <mergeCells count="48">
-    <mergeCell ref="E1:N1"/>
-    <mergeCell ref="S1:AB1"/>
-    <mergeCell ref="AG1:AP1"/>
-    <mergeCell ref="AU1:BD1"/>
-    <mergeCell ref="BI1:BR1"/>
-    <mergeCell ref="BW1:CF1"/>
-    <mergeCell ref="CK1:CT1"/>
-    <mergeCell ref="CY1:DH1"/>
-    <mergeCell ref="DM1:DV1"/>
-    <mergeCell ref="EA1:EJ1"/>
+    <mergeCell ref="FE2:FH2"/>
+    <mergeCell ref="FI2:FL2"/>
+    <mergeCell ref="EG2:EJ2"/>
+    <mergeCell ref="EO2:EP2"/>
+    <mergeCell ref="EQ2:ET2"/>
+    <mergeCell ref="EU2:EX2"/>
+    <mergeCell ref="FC2:FD2"/>
+    <mergeCell ref="DM2:DN2"/>
+    <mergeCell ref="DO2:DR2"/>
+    <mergeCell ref="DS2:DV2"/>
+    <mergeCell ref="EA2:EB2"/>
+    <mergeCell ref="EC2:EF2"/>
+    <mergeCell ref="CM2:CP2"/>
+    <mergeCell ref="CQ2:CT2"/>
+    <mergeCell ref="CY2:CZ2"/>
+    <mergeCell ref="DA2:DD2"/>
+    <mergeCell ref="DE2:DH2"/>
+    <mergeCell ref="BO2:BR2"/>
+    <mergeCell ref="BW2:BX2"/>
+    <mergeCell ref="BY2:CB2"/>
+    <mergeCell ref="CC2:CF2"/>
+    <mergeCell ref="CK2:CL2"/>
     <mergeCell ref="EO1:EX1"/>
     <mergeCell ref="FC1:FL1"/>
     <mergeCell ref="E2:F2"/>
@@ -5422,28 +5435,16 @@
     <mergeCell ref="BA2:BD2"/>
     <mergeCell ref="BI2:BJ2"/>
     <mergeCell ref="BK2:BN2"/>
-    <mergeCell ref="BO2:BR2"/>
-    <mergeCell ref="BW2:BX2"/>
-    <mergeCell ref="BY2:CB2"/>
-    <mergeCell ref="CC2:CF2"/>
-    <mergeCell ref="CK2:CL2"/>
-    <mergeCell ref="CM2:CP2"/>
-    <mergeCell ref="CQ2:CT2"/>
-    <mergeCell ref="CY2:CZ2"/>
-    <mergeCell ref="DA2:DD2"/>
-    <mergeCell ref="DE2:DH2"/>
-    <mergeCell ref="DM2:DN2"/>
-    <mergeCell ref="DO2:DR2"/>
-    <mergeCell ref="DS2:DV2"/>
-    <mergeCell ref="EA2:EB2"/>
-    <mergeCell ref="EC2:EF2"/>
-    <mergeCell ref="FE2:FH2"/>
-    <mergeCell ref="FI2:FL2"/>
-    <mergeCell ref="EG2:EJ2"/>
-    <mergeCell ref="EO2:EP2"/>
-    <mergeCell ref="EQ2:ET2"/>
-    <mergeCell ref="EU2:EX2"/>
-    <mergeCell ref="FC2:FD2"/>
+    <mergeCell ref="BW1:CF1"/>
+    <mergeCell ref="CK1:CT1"/>
+    <mergeCell ref="CY1:DH1"/>
+    <mergeCell ref="DM1:DV1"/>
+    <mergeCell ref="EA1:EJ1"/>
+    <mergeCell ref="E1:N1"/>
+    <mergeCell ref="S1:AB1"/>
+    <mergeCell ref="AG1:AP1"/>
+    <mergeCell ref="AU1:BD1"/>
+    <mergeCell ref="BI1:BR1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>